<commit_message>
update wrong Gemma 4 e4b results and tests for qwen 3.5 9b
</commit_message>
<xml_diff>
--- a/results/compiled results.xlsx
+++ b/results/compiled results.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elish\Desktop\Aims Project\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E93E0A5D-474B-46DC-B895-D8C2846DBBFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42F5BE61-90B5-4E26-85D8-CB9F0DEA751B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic results" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="7" r:id="rId2"/>
+    <sheet name="Model details" sheetId="7" r:id="rId2"/>
     <sheet name="Multiple safety results" sheetId="4" r:id="rId3"/>
     <sheet name="Simple cluttered resutls" sheetId="5" r:id="rId4"/>
     <sheet name="Complex cluttered results" sheetId="6" r:id="rId5"/>
@@ -564,7 +564,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -737,39 +737,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -800,6 +769,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1171,26 +1164,26 @@
       <c r="A2" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="67" t="s">
+      <c r="C2" s="78"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="67"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="67" t="s">
+      <c r="F2" s="78"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="66" t="s">
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
       <c r="N2" s="1" t="s">
         <v>37</v>
       </c>
@@ -2116,26 +2109,26 @@
       <c r="A27" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B27" s="66" t="s">
+      <c r="B27" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="67"/>
-      <c r="D27" s="68"/>
-      <c r="E27" s="67" t="s">
+      <c r="C27" s="78"/>
+      <c r="D27" s="79"/>
+      <c r="E27" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F27" s="67"/>
-      <c r="G27" s="68"/>
-      <c r="H27" s="67" t="s">
+      <c r="F27" s="78"/>
+      <c r="G27" s="79"/>
+      <c r="H27" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I27" s="67"/>
-      <c r="J27" s="67"/>
-      <c r="K27" s="66" t="s">
+      <c r="I27" s="78"/>
+      <c r="J27" s="78"/>
+      <c r="K27" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L27" s="67"/>
-      <c r="M27" s="67"/>
+      <c r="L27" s="78"/>
+      <c r="M27" s="78"/>
       <c r="O27" s="34" t="s">
         <v>34</v>
       </c>
@@ -2885,26 +2878,26 @@
       <c r="A47" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B47" s="66" t="s">
+      <c r="B47" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C47" s="67"/>
-      <c r="D47" s="68"/>
-      <c r="E47" s="67" t="s">
+      <c r="C47" s="78"/>
+      <c r="D47" s="79"/>
+      <c r="E47" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F47" s="67"/>
-      <c r="G47" s="68"/>
-      <c r="H47" s="67" t="s">
+      <c r="F47" s="78"/>
+      <c r="G47" s="79"/>
+      <c r="H47" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I47" s="67"/>
-      <c r="J47" s="67"/>
-      <c r="K47" s="66" t="s">
+      <c r="I47" s="78"/>
+      <c r="J47" s="78"/>
+      <c r="K47" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L47" s="67"/>
-      <c r="M47" s="67"/>
+      <c r="L47" s="78"/>
+      <c r="M47" s="78"/>
       <c r="T47" s="31"/>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.3">
@@ -3658,26 +3651,26 @@
       <c r="A70" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B70" s="66" t="s">
+      <c r="B70" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C70" s="67"/>
-      <c r="D70" s="68"/>
-      <c r="E70" s="67" t="s">
+      <c r="C70" s="78"/>
+      <c r="D70" s="79"/>
+      <c r="E70" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F70" s="67"/>
-      <c r="G70" s="68"/>
-      <c r="H70" s="67" t="s">
+      <c r="F70" s="78"/>
+      <c r="G70" s="79"/>
+      <c r="H70" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I70" s="67"/>
-      <c r="J70" s="67"/>
-      <c r="K70" s="66" t="s">
+      <c r="I70" s="78"/>
+      <c r="J70" s="78"/>
+      <c r="K70" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L70" s="67"/>
-      <c r="M70" s="67"/>
+      <c r="L70" s="78"/>
+      <c r="M70" s="78"/>
       <c r="T70" s="31"/>
     </row>
     <row r="71" spans="1:27" x14ac:dyDescent="0.3">
@@ -4495,6 +4488,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B70:D70"/>
+    <mergeCell ref="E70:G70"/>
+    <mergeCell ref="H70:J70"/>
+    <mergeCell ref="K70:M70"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="E47:G47"/>
+    <mergeCell ref="H47:J47"/>
+    <mergeCell ref="K47:M47"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -4503,14 +4504,6 @@
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="H27:J27"/>
     <mergeCell ref="K27:M27"/>
-    <mergeCell ref="B70:D70"/>
-    <mergeCell ref="E70:G70"/>
-    <mergeCell ref="H70:J70"/>
-    <mergeCell ref="K70:M70"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="E47:G47"/>
-    <mergeCell ref="H47:J47"/>
-    <mergeCell ref="K47:M47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4518,232 +4511,196 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333A2C69-865F-4E01-AA50-D93BFCA52E39}">
-  <dimension ref="E15:K26"/>
+  <dimension ref="F16:K24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="13.6640625" customWidth="1"/>
     <col min="7" max="7" width="19.109375" customWidth="1"/>
-    <col min="8" max="8" width="8.5546875" style="74" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" style="74" customWidth="1"/>
+    <col min="8" max="8" width="8.5546875" style="66" customWidth="1"/>
+    <col min="9" max="9" width="7.44140625" style="66" customWidth="1"/>
     <col min="10" max="10" width="17.44140625" customWidth="1"/>
     <col min="11" max="11" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="15" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E15" s="75"/>
-      <c r="F15" s="75"/>
-      <c r="G15" s="75"/>
-      <c r="H15" s="76"/>
-      <c r="I15" s="76"/>
-      <c r="J15" s="75"/>
-      <c r="K15" s="75"/>
-    </row>
-    <row r="16" spans="5:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="E16" s="75"/>
+    <row r="16" spans="6:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="F16" s="48" t="s">
         <v>63</v>
       </c>
-      <c r="G16" s="85" t="s">
+      <c r="G16" s="74" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="83" t="s">
+      <c r="H16" s="72" t="s">
         <v>71</v>
       </c>
-      <c r="I16" s="86" t="s">
+      <c r="I16" s="75" t="s">
         <v>74</v>
       </c>
-      <c r="J16" s="85" t="s">
+      <c r="J16" s="74" t="s">
         <v>79</v>
       </c>
       <c r="K16" s="65" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="17" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E17" s="75"/>
+    <row r="17" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F17" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="G17" s="84" t="s">
+      <c r="G17" s="73" t="s">
         <v>67</v>
       </c>
-      <c r="H17" s="83" t="s">
+      <c r="H17" s="72" t="s">
         <v>81</v>
       </c>
-      <c r="I17" s="87" t="s">
+      <c r="I17" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="J17" s="82" t="s">
+      <c r="J17" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="K17" s="84" t="s">
+      <c r="K17" s="73" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E18" s="75"/>
+    <row r="18" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F18" s="12" t="s">
         <v>76</v>
       </c>
       <c r="G18" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="H18" s="81" t="s">
+      <c r="H18" s="70" t="s">
         <v>81</v>
       </c>
-      <c r="I18" s="81" t="s">
+      <c r="I18" s="70" t="s">
         <v>68</v>
       </c>
-      <c r="J18" s="79" t="s">
+      <c r="J18" s="68" t="s">
         <v>83</v>
       </c>
-      <c r="K18" s="77" t="s">
+      <c r="K18" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E19" s="75"/>
+    <row r="19" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F19" s="5" t="s">
         <v>76</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="H19" s="80" t="s">
+      <c r="H19" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="I19" s="80" t="s">
+      <c r="I19" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="J19" s="78" t="s">
+      <c r="J19" s="67" t="s">
         <v>83</v>
       </c>
       <c r="K19" s="13" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E20" s="75"/>
+    <row r="20" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F20" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="G20" s="79" t="s">
+      <c r="G20" s="68" t="s">
         <v>67</v>
       </c>
-      <c r="H20" s="81" t="s">
+      <c r="H20" s="70" t="s">
         <v>72</v>
       </c>
-      <c r="I20" s="81" t="s">
+      <c r="I20" s="70" t="s">
         <v>69</v>
       </c>
-      <c r="J20" s="79" t="s">
+      <c r="J20" s="68" t="s">
         <v>83</v>
       </c>
-      <c r="K20" s="77" t="s">
+      <c r="K20" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E21" s="75"/>
+    <row r="21" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F21" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G21" s="78" t="s">
+      <c r="G21" s="67" t="s">
         <v>66</v>
       </c>
-      <c r="H21" s="80" t="s">
+      <c r="H21" s="69" t="s">
         <v>86</v>
       </c>
-      <c r="I21" s="80" t="s">
+      <c r="I21" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="J21" s="78" t="s">
+      <c r="J21" s="67" t="s">
         <v>83</v>
       </c>
       <c r="K21" s="13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E22" s="75"/>
+    <row r="22" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F22" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="G22" s="79" t="s">
+      <c r="G22" s="68" t="s">
         <v>67</v>
       </c>
-      <c r="H22" s="81" t="s">
+      <c r="H22" s="70" t="s">
         <v>84</v>
       </c>
-      <c r="I22" s="81" t="s">
+      <c r="I22" s="70" t="s">
         <v>70</v>
       </c>
-      <c r="J22" s="79" t="s">
+      <c r="J22" s="68" t="s">
         <v>83</v>
       </c>
-      <c r="K22" s="77" t="s">
+      <c r="K22" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E23" s="75"/>
+    <row r="23" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F23" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="G23" s="79" t="s">
+      <c r="G23" s="68" t="s">
         <v>65</v>
       </c>
-      <c r="H23" s="81" t="s">
+      <c r="H23" s="70" t="s">
         <v>85</v>
       </c>
-      <c r="I23" s="81" t="s">
+      <c r="I23" s="70" t="s">
         <v>70</v>
       </c>
-      <c r="J23" s="79" t="s">
+      <c r="J23" s="68" t="s">
         <v>83</v>
       </c>
-      <c r="K23" s="77" t="s">
+      <c r="K23" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="24" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E24" s="75"/>
+    <row r="24" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F24" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G24" s="78" t="s">
+      <c r="G24" s="67" t="s">
         <v>65</v>
       </c>
-      <c r="H24" s="80" t="s">
+      <c r="H24" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="I24" s="80" t="s">
+      <c r="I24" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="J24" s="78" t="s">
+      <c r="J24" s="67" t="s">
         <v>83</v>
       </c>
       <c r="K24" s="13" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="25" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E25" s="75"/>
-      <c r="F25" s="75"/>
-      <c r="G25" s="75"/>
-      <c r="H25" s="76"/>
-      <c r="I25" s="76"/>
-      <c r="J25" s="75"/>
-      <c r="K25" s="75"/>
-    </row>
-    <row r="26" spans="5:11" x14ac:dyDescent="0.3">
-      <c r="E26" s="75"/>
-      <c r="F26" s="75"/>
-      <c r="G26" s="75"/>
-      <c r="H26" s="76"/>
-      <c r="I26" s="76"/>
-      <c r="J26" s="75"/>
-      <c r="K26" s="75"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -4780,26 +4737,26 @@
       <c r="A2" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="67" t="s">
+      <c r="C2" s="78"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="67"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="67" t="s">
+      <c r="F2" s="78"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="66" t="s">
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -5398,43 +5355,43 @@
         <v>58</v>
       </c>
       <c r="P17" s="3">
-        <v>0.20094616602850901</v>
+        <v>0.36366496008710802</v>
       </c>
       <c r="Q17" s="3">
-        <v>0.107460022996064</v>
+        <v>8.5103341494056503E-2</v>
       </c>
       <c r="R17" s="3">
-        <v>0.20170607435510901</v>
+        <v>0.36356107891046802</v>
       </c>
       <c r="S17" s="43">
-        <v>0.108864617481995</v>
+        <v>8.5107195582413003E-2</v>
       </c>
       <c r="T17" s="31">
         <v>0</v>
       </c>
       <c r="U17" s="50">
-        <v>0</v>
+        <v>87.1</v>
       </c>
       <c r="V17" s="3">
-        <v>4.7640653619619E-2</v>
+        <v>5.6548667764616201E-2</v>
       </c>
       <c r="W17" s="43">
-        <v>5.6548667764616201E-2</v>
+        <v>0</v>
       </c>
       <c r="X17" s="3">
-        <v>2.3199999999999901E-2</v>
+        <v>0.156799999999999</v>
       </c>
       <c r="Y17" s="43">
-        <v>2.619904</v>
+        <v>0.37631999999999999</v>
       </c>
       <c r="Z17" s="31">
-        <v>98.918181818181793</v>
+        <v>100</v>
       </c>
       <c r="AA17" s="31">
-        <v>10.881</v>
+        <v>11</v>
       </c>
       <c r="AB17" s="31">
-        <v>7108.14468373205</v>
+        <v>4079.1357275988898</v>
       </c>
       <c r="AD17" s="3">
         <v>5.6548667764616201E-2</v>
@@ -5652,26 +5609,26 @@
       <c r="A24" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B24" s="66" t="s">
+      <c r="B24" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="67"/>
-      <c r="D24" s="68"/>
-      <c r="E24" s="67" t="s">
+      <c r="C24" s="78"/>
+      <c r="D24" s="79"/>
+      <c r="E24" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F24" s="67"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="67" t="s">
+      <c r="F24" s="78"/>
+      <c r="G24" s="79"/>
+      <c r="H24" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I24" s="67"/>
-      <c r="J24" s="67"/>
-      <c r="K24" s="66" t="s">
+      <c r="I24" s="78"/>
+      <c r="J24" s="78"/>
+      <c r="K24" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L24" s="67"/>
-      <c r="M24" s="67"/>
+      <c r="L24" s="78"/>
+      <c r="M24" s="78"/>
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
@@ -6454,26 +6411,26 @@
       <c r="A44" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="66" t="s">
+      <c r="B44" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="67"/>
-      <c r="D44" s="68"/>
-      <c r="E44" s="67" t="s">
+      <c r="C44" s="78"/>
+      <c r="D44" s="79"/>
+      <c r="E44" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="67"/>
-      <c r="G44" s="68"/>
-      <c r="H44" s="67" t="s">
+      <c r="F44" s="78"/>
+      <c r="G44" s="79"/>
+      <c r="H44" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I44" s="67"/>
-      <c r="J44" s="67"/>
-      <c r="K44" s="66" t="s">
+      <c r="I44" s="78"/>
+      <c r="J44" s="78"/>
+      <c r="K44" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="67"/>
-      <c r="M44" s="67"/>
+      <c r="L44" s="78"/>
+      <c r="M44" s="78"/>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -7256,26 +7213,26 @@
       <c r="A65" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="69" t="s">
+      <c r="B65" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="C65" s="70"/>
-      <c r="D65" s="71"/>
-      <c r="E65" s="72" t="s">
+      <c r="C65" s="81"/>
+      <c r="D65" s="82"/>
+      <c r="E65" s="83" t="s">
         <v>25</v>
       </c>
-      <c r="F65" s="70"/>
-      <c r="G65" s="71"/>
-      <c r="H65" s="72" t="s">
+      <c r="F65" s="81"/>
+      <c r="G65" s="82"/>
+      <c r="H65" s="83" t="s">
         <v>26</v>
       </c>
-      <c r="I65" s="70"/>
-      <c r="J65" s="73"/>
-      <c r="K65" s="69" t="s">
+      <c r="I65" s="81"/>
+      <c r="J65" s="84"/>
+      <c r="K65" s="80" t="s">
         <v>27</v>
       </c>
-      <c r="L65" s="70"/>
-      <c r="M65" s="70"/>
+      <c r="L65" s="81"/>
+      <c r="M65" s="81"/>
       <c r="N65" s="21"/>
       <c r="O65" s="21"/>
     </row>
@@ -8129,6 +8086,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="E65:G65"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="K65:M65"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -8137,14 +8102,6 @@
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="H24:J24"/>
     <mergeCell ref="K24:M24"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="E65:G65"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="K65:M65"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="K44:M44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8180,26 +8137,26 @@
       <c r="A2" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="67" t="s">
+      <c r="C2" s="78"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="67"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="67" t="s">
+      <c r="F2" s="78"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="66" t="s">
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -8904,26 +8861,26 @@
       <c r="A23" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="67"/>
-      <c r="D23" s="68"/>
-      <c r="E23" s="67" t="s">
+      <c r="C23" s="78"/>
+      <c r="D23" s="79"/>
+      <c r="E23" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="67"/>
-      <c r="G23" s="68"/>
-      <c r="H23" s="67" t="s">
+      <c r="F23" s="78"/>
+      <c r="G23" s="79"/>
+      <c r="H23" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I23" s="67"/>
-      <c r="J23" s="67"/>
-      <c r="K23" s="66" t="s">
+      <c r="I23" s="78"/>
+      <c r="J23" s="78"/>
+      <c r="K23" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L23" s="67"/>
-      <c r="M23" s="67"/>
+      <c r="L23" s="78"/>
+      <c r="M23" s="78"/>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -9581,26 +9538,26 @@
       <c r="A44" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="66" t="s">
+      <c r="B44" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="67"/>
-      <c r="D44" s="68"/>
-      <c r="E44" s="67" t="s">
+      <c r="C44" s="78"/>
+      <c r="D44" s="79"/>
+      <c r="E44" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="67"/>
-      <c r="G44" s="68"/>
-      <c r="H44" s="67" t="s">
+      <c r="F44" s="78"/>
+      <c r="G44" s="79"/>
+      <c r="H44" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I44" s="67"/>
-      <c r="J44" s="67"/>
-      <c r="K44" s="66" t="s">
+      <c r="I44" s="78"/>
+      <c r="J44" s="78"/>
+      <c r="K44" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="67"/>
-      <c r="M44" s="67"/>
+      <c r="L44" s="78"/>
+      <c r="M44" s="78"/>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -10258,26 +10215,26 @@
       <c r="A64" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B64" s="69" t="s">
+      <c r="B64" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="C64" s="70"/>
-      <c r="D64" s="71"/>
-      <c r="E64" s="72" t="s">
+      <c r="C64" s="81"/>
+      <c r="D64" s="82"/>
+      <c r="E64" s="83" t="s">
         <v>25</v>
       </c>
-      <c r="F64" s="70"/>
-      <c r="G64" s="71"/>
-      <c r="H64" s="72" t="s">
+      <c r="F64" s="81"/>
+      <c r="G64" s="82"/>
+      <c r="H64" s="83" t="s">
         <v>26</v>
       </c>
-      <c r="I64" s="70"/>
-      <c r="J64" s="73"/>
-      <c r="K64" s="69" t="s">
+      <c r="I64" s="81"/>
+      <c r="J64" s="84"/>
+      <c r="K64" s="80" t="s">
         <v>27</v>
       </c>
-      <c r="L64" s="70"/>
-      <c r="M64" s="70"/>
+      <c r="L64" s="81"/>
+      <c r="M64" s="81"/>
       <c r="N64" s="21"/>
       <c r="O64" s="56"/>
     </row>
@@ -11131,6 +11088,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="E64:G64"/>
+    <mergeCell ref="H64:J64"/>
+    <mergeCell ref="K64:M64"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -11139,14 +11104,6 @@
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:J23"/>
     <mergeCell ref="K23:M23"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="E64:G64"/>
-    <mergeCell ref="H64:J64"/>
-    <mergeCell ref="K64:M64"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11183,26 +11140,26 @@
       <c r="A2" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="67" t="s">
+      <c r="C2" s="78"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="67"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="67" t="s">
+      <c r="F2" s="78"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="66" t="s">
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -11907,26 +11864,26 @@
       <c r="A23" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="67"/>
-      <c r="D23" s="68"/>
-      <c r="E23" s="67" t="s">
+      <c r="C23" s="78"/>
+      <c r="D23" s="79"/>
+      <c r="E23" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="67"/>
-      <c r="G23" s="68"/>
-      <c r="H23" s="67" t="s">
+      <c r="F23" s="78"/>
+      <c r="G23" s="79"/>
+      <c r="H23" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I23" s="67"/>
-      <c r="J23" s="67"/>
-      <c r="K23" s="66" t="s">
+      <c r="I23" s="78"/>
+      <c r="J23" s="78"/>
+      <c r="K23" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L23" s="67"/>
-      <c r="M23" s="67"/>
+      <c r="L23" s="78"/>
+      <c r="M23" s="78"/>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -12584,26 +12541,26 @@
       <c r="A44" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="66" t="s">
+      <c r="B44" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="67"/>
-      <c r="D44" s="68"/>
-      <c r="E44" s="67" t="s">
+      <c r="C44" s="78"/>
+      <c r="D44" s="79"/>
+      <c r="E44" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="67"/>
-      <c r="G44" s="68"/>
-      <c r="H44" s="67" t="s">
+      <c r="F44" s="78"/>
+      <c r="G44" s="79"/>
+      <c r="H44" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I44" s="67"/>
-      <c r="J44" s="67"/>
-      <c r="K44" s="66" t="s">
+      <c r="I44" s="78"/>
+      <c r="J44" s="78"/>
+      <c r="K44" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="67"/>
-      <c r="M44" s="67"/>
+      <c r="L44" s="78"/>
+      <c r="M44" s="78"/>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -13192,26 +13149,26 @@
       <c r="A65" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="69" t="s">
+      <c r="B65" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="C65" s="70"/>
-      <c r="D65" s="71"/>
-      <c r="E65" s="72" t="s">
+      <c r="C65" s="81"/>
+      <c r="D65" s="82"/>
+      <c r="E65" s="83" t="s">
         <v>25</v>
       </c>
-      <c r="F65" s="70"/>
-      <c r="G65" s="71"/>
-      <c r="H65" s="72" t="s">
+      <c r="F65" s="81"/>
+      <c r="G65" s="82"/>
+      <c r="H65" s="83" t="s">
         <v>26</v>
       </c>
-      <c r="I65" s="70"/>
-      <c r="J65" s="73"/>
-      <c r="K65" s="69" t="s">
+      <c r="I65" s="81"/>
+      <c r="J65" s="84"/>
+      <c r="K65" s="80" t="s">
         <v>27</v>
       </c>
-      <c r="L65" s="70"/>
-      <c r="M65" s="70"/>
+      <c r="L65" s="81"/>
+      <c r="M65" s="81"/>
       <c r="N65" s="21"/>
       <c r="O65" s="56"/>
     </row>
@@ -14065,6 +14022,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="E65:G65"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="K65:M65"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -14073,14 +14038,6 @@
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:J23"/>
     <mergeCell ref="K23:M23"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="E65:G65"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="K65:M65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>